<commit_message>
feat(boutique): apply new euro prices from prix.csv
36 of 42 titles updated. Six rows still carry old CAD prices in the
price list and were left unchanged.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/prix/prix.xlsx
+++ b/prix/prix.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fabricemaudieu/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fabricemaudieu/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96230006-BC22-CD48-9A31-7245B676493E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C72FE58-8FAC-D04B-911D-EF605A7CB094}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="28800" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Catalogue complet" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="103">
   <si>
     <t>Couverture</t>
   </si>
@@ -34,9 +34,6 @@
     <t>Prix (CAD)</t>
   </si>
   <si>
-    <t>SKU</t>
-  </si>
-  <si>
     <t>Description</t>
   </si>
   <si>
@@ -49,279 +46,108 @@
     <t>Précepte sur Précepte</t>
   </si>
   <si>
-    <t>$24.75</t>
-  </si>
-  <si>
-    <t>70159</t>
-  </si>
-  <si>
     <t>Voir le produit</t>
   </si>
   <si>
     <t>2 Timothée — Précepte sur Précepte</t>
   </si>
   <si>
-    <t>$29.25</t>
-  </si>
-  <si>
-    <t>70158</t>
-  </si>
-  <si>
     <t>Esdras et Aggée — Précepte sur Précepte</t>
   </si>
   <si>
-    <t>$15.99</t>
-  </si>
-  <si>
-    <t>70714</t>
-  </si>
-  <si>
     <t>Genèse Partie 1 — Précepte sur Précepte</t>
   </si>
   <si>
-    <t>70860</t>
-  </si>
-  <si>
     <t>Genèse Partie 2 — Précepte sur Précepte</t>
   </si>
   <si>
-    <t>$21.99</t>
-  </si>
-  <si>
-    <t>70859</t>
-  </si>
-  <si>
     <t>Genèse Partie 3 — Précepte sur Précepte</t>
   </si>
   <si>
-    <t>70858</t>
-  </si>
-  <si>
     <t>L'Alliance — Précepte sur Précepte</t>
   </si>
   <si>
-    <t>$18.99</t>
-  </si>
-  <si>
-    <t>70861</t>
-  </si>
-  <si>
     <t>Romains Partie 1 (ch.1–5) — Précepte sur Précepte</t>
   </si>
   <si>
-    <t>$32.99</t>
-  </si>
-  <si>
-    <t>70753</t>
-  </si>
-  <si>
     <t>Romains Partie 2 (ch.6–8) — Précepte sur Précepte</t>
   </si>
   <si>
-    <t>$24.99</t>
-  </si>
-  <si>
-    <t>70754</t>
-  </si>
-  <si>
     <t>Romains Partie 3 (ch.9–11) — Précepte sur Précepte</t>
   </si>
   <si>
-    <t>70822</t>
-  </si>
-  <si>
     <t>Romains Partie 4 (ch.12–16) — Précepte sur Précepte</t>
   </si>
   <si>
-    <t>70823</t>
-  </si>
-  <si>
     <t>Tite — Précepte sur Précepte</t>
   </si>
   <si>
     <t>$11.99</t>
   </si>
   <si>
-    <t>70759</t>
-  </si>
-  <si>
     <t>Bâtir un mariage qui fructifie vraiment</t>
   </si>
   <si>
     <t>Série 40 minutes</t>
   </si>
   <si>
-    <t>22251</t>
-  </si>
-  <si>
     <t>Comment faire des choix que vous ne regretterez pas</t>
   </si>
   <si>
-    <t>22006</t>
-  </si>
-  <si>
-    <t>Every day you face choices. Discover what God's Word says about making decisions you will never regret.</t>
-  </si>
-  <si>
     <t>Comment savoir que Dieu est votre Père ?</t>
   </si>
   <si>
-    <t>21986</t>
-  </si>
-  <si>
-    <t>How do you know that God is truly your Father? Explore the assurance of salvation and what it means to be a child of God.</t>
-  </si>
-  <si>
     <t>Enflammez votre passion pour Dieu</t>
   </si>
   <si>
-    <t>22222</t>
-  </si>
-  <si>
-    <t>Rekindle your passion for God. This 40-minute study shows you how to pursue Him with your whole heart.</t>
-  </si>
-  <si>
     <t>Entretenir une relation réelle avec Dieu</t>
   </si>
   <si>
-    <t>21987</t>
-  </si>
-  <si>
-    <t>What does it look like to have a genuine, growing relationship with God? This 40-minute study gives you practical and biblical answers.</t>
-  </si>
-  <si>
     <t>Être un disciple : ce qu'il en coûte vraiment</t>
   </si>
   <si>
-    <t>22005</t>
-  </si>
-  <si>
-    <t>What does it really cost to be a disciple of Jesus? This honest 40-minute study examines the true demands of following Christ.</t>
-  </si>
-  <si>
     <t>Jésus : à l'écoute de sa voix</t>
   </si>
   <si>
-    <t>22242</t>
-  </si>
-  <si>
-    <t>Are you listening for the voice of Jesus? This 40-minute study helps you recognise and respond to His call.</t>
-  </si>
-  <si>
     <t>Jésus : comprendre sa mort et sa résurrection</t>
   </si>
   <si>
-    <t>22252</t>
-  </si>
-  <si>
-    <t>Why did Jesus die? What does the resurrection mean for you? This 40-minute study gives clear, life-changing answers.</t>
-  </si>
-  <si>
     <t>Jésus : faire l'expérience de son toucher</t>
   </si>
   <si>
-    <t>22241</t>
-  </si>
-  <si>
-    <t>Jesus touched lepers, the broken, and the outcasts. This 40-minute study invites you to experience His transforming touch.</t>
-  </si>
-  <si>
     <t>Le ciel, l'enfer et la vie après la mort</t>
   </si>
   <si>
-    <t>22229</t>
-  </si>
-  <si>
-    <t>What does the Bible say about heaven, hell, and life after death? This 40-minute study gives you clear, biblical answers.</t>
-  </si>
-  <si>
     <t>Libéré de l'emprise de la peur</t>
   </si>
   <si>
-    <t>22280</t>
-  </si>
-  <si>
-    <t>Fear has a grip on many people. Discover what God's Word says and how you can be freed from the power of fear.</t>
-  </si>
-  <si>
     <t>Mener une vie d'adoration authentique</t>
   </si>
   <si>
-    <t>22230</t>
-  </si>
-  <si>
-    <t>What does authentic worship look like? This 40-minute study explores what it means to truly glorify God in every area of life.</t>
-  </si>
-  <si>
     <t>Pardonner : briser l'emprise du passé</t>
   </si>
   <si>
-    <t>22228</t>
-  </si>
-  <si>
-    <t>Forgiveness can break the power of the past. This 40-minute study shows you how to forgive as God has forgiven you.</t>
-  </si>
-  <si>
     <t>Abraham, le vaillant explorateur de Dieu</t>
   </si>
   <si>
     <t>Découvrir par toi-même</t>
   </si>
   <si>
-    <t>22227</t>
-  </si>
-  <si>
-    <t>Journey with Abraham – the father of faith. Discover how God called him, tested him, and kept His promises. An inspiring study for children ages 7–12.</t>
-  </si>
-  <si>
     <t>Déterrons le passé (Genèse 3–11)</t>
   </si>
   <si>
-    <t>22007</t>
-  </si>
-  <si>
-    <t>Dig into Genesis 3–11 and uncover the origins of sin, the flood, and the nations. A discovery study for children ages 7–12.</t>
-  </si>
-  <si>
     <t>Jésus – puissance incroyable, amour incroyable</t>
   </si>
   <si>
-    <t>$14.99</t>
-  </si>
-  <si>
-    <t>22261</t>
-  </si>
-  <si>
-    <t>John 11–16: Witness the incredible power and love of Jesus as He raises the dead, washes feet, and promises the Holy Spirit.</t>
-  </si>
-  <si>
     <t>Jésus sous les réflecteurs (Jean 1–10)</t>
   </si>
   <si>
-    <t>22260</t>
-  </si>
-  <si>
-    <t>John 1–10: Who is Jesus? This discovery study for children 7–12 puts Jesus in the spotlight and lets God's Word speak for itself.</t>
-  </si>
-  <si>
     <t>Jésus – vers l'éternité et au-delà (Jean 17–21)</t>
   </si>
   <si>
-    <t>22262</t>
-  </si>
-  <si>
-    <t>John 17–21: Follow Jesus to the cross, the empty tomb, and beyond. A children's discovery study on the culmination of Jesus' ministry.</t>
-  </si>
-  <si>
     <t>L'extraordinaire création de Dieu (Genèse 1–2)</t>
   </si>
   <si>
-    <t>22226</t>
-  </si>
-  <si>
-    <t>Genesis 1–2: Explore the wonder of God's creation with this discovery study designed for children ages 7–12.</t>
-  </si>
-  <si>
     <t>Dieu, es-tu là ? T'intéresses-tu à moi ?</t>
   </si>
   <si>
@@ -331,105 +157,42 @@
     <t>$17.99</t>
   </si>
   <si>
-    <t>21369</t>
-  </si>
-  <si>
-    <t>Is God really there? Does He care about you? Does He know you? This foundational study addresses life's most important questions.</t>
-  </si>
-  <si>
     <t>Seigneur, enseigne-moi à étudier la Bible</t>
   </si>
   <si>
     <t>$16.99</t>
   </si>
   <si>
-    <t>22210</t>
-  </si>
-  <si>
-    <t>A 28-day journey to learn the Precept inductive Bible study method — Observe, Interpret, and Apply God's Word for yourself.</t>
-  </si>
-  <si>
     <t>Seigneur, enseigne-moi à prier en 28 jours</t>
   </si>
   <si>
-    <t>21279</t>
-  </si>
-  <si>
-    <t>In 28 days, learn to pray through God's Word. Discover the principles of prayer as taught throughout Scripture.</t>
-  </si>
-  <si>
     <t>Seigneur, j'ai besoin de réponses</t>
   </si>
   <si>
-    <t>22231</t>
-  </si>
-  <si>
-    <t>When life raises hard questions, God's Word has answers. This study addresses some of the most challenging questions believers face.</t>
-  </si>
-  <si>
     <t>Seigneur, je veux te connaître</t>
   </si>
   <si>
-    <t>$19.99</t>
-  </si>
-  <si>
-    <t>22265</t>
-  </si>
-  <si>
-    <t>An in-depth study of the names and character of God. Come to know Him as He truly is, not just as you imagine Him to be.</t>
-  </si>
-  <si>
     <t>Choisir la victoire – Triompher de la défaite</t>
   </si>
   <si>
     <t>Collection Études inductives</t>
   </si>
   <si>
-    <t>21476</t>
-  </si>
-  <si>
-    <t>Study the books of Joshua, Judges, and Ruth and learn how to choose victory over defeat in your daily walk with God.</t>
-  </si>
-  <si>
     <t>Enfin libéré de l'esclavage ! (Galates, Éphésiens)</t>
   </si>
   <si>
-    <t>21267</t>
-  </si>
-  <si>
-    <t>A study of Galatians and Ephesians. Discover the freedom that Christ won for you and how to live free from the bondage of sin.</t>
-  </si>
-  <si>
     <t>Enseigne-moi tes voies (Pentateuque)</t>
   </si>
   <si>
     <t>$13.99</t>
   </si>
   <si>
-    <t>22263</t>
-  </si>
-  <si>
-    <t>An inductive study through Genesis, Exodus, Leviticus, Numbers, and Deuteronomy. Learn God's ways and how to walk in them.</t>
-  </si>
-  <si>
     <t>L'appel à suivre Jésus (Luc)</t>
   </si>
   <si>
-    <t>21477</t>
-  </si>
-  <si>
-    <t>An inductive study through the Gospel of Luke. Discover what it means to answer Jesus' call to follow Him.</t>
-  </si>
-  <si>
     <t>La clé pour vivre par la Foi (Hébreux)</t>
   </si>
   <si>
-    <t>21478</t>
-  </si>
-  <si>
-    <t>Hebrews: What is faith and how do you live by it? Study the great cloud of witnesses and the superiority of Christ.</t>
-  </si>
-  <si>
     <t>Philippiens — Saisir et Agir</t>
   </si>
   <si>
@@ -437,12 +200,6 @@
   </si>
   <si>
     <t>$22.99</t>
-  </si>
-  <si>
-    <t>70912</t>
-  </si>
-  <si>
-    <t>A Saisir et Agir (Seize and Apply) study of Philippians with approximately 3 hours of homework per week.</t>
   </si>
   <si>
     <t>Êtes-vous un exemple pour les autres ? Découvrez les principes d'une vie chrétienne exemplaire. Comprenez la réalité du combat spirituel suscité par la présence de l'Évangile dans le monde, ainsi que l'enlèvement de l'Église, le secours ultime que Dieu réserve à son peuple.</t>
@@ -491,13 +248,108 @@
   <si>
     <t>Découvrez ce que Dieu dit au sujet du mariage et comment construire une relation qui s’épanouit véritablement.
 Une étude concise de 40 minutes, sans devoirs à faire.</t>
+  </si>
+  <si>
+    <t>Chaque jour, vous devez faire des choix. Découvrez ce que dit la Parole de Dieu sur la manière de prendre des décisions que vous ne regretterez jamais.</t>
+  </si>
+  <si>
+    <t>Comment savez-vous que Dieu est véritablement votre Père ? Découvrez l'assurance du salut et ce que signifie être un enfant de Dieu.</t>
+  </si>
+  <si>
+    <t>Ravivez votre passion pour Dieu. Cette étude de 40 minutes vous montre comment Le rechercher de tout votre cœur.</t>
+  </si>
+  <si>
+    <t>À quoi ressemble une relation authentique et grandissante avec Dieu ? Cette étude de 40 minutes vous apporte des réponses concrètes et bibliques.</t>
+  </si>
+  <si>
+    <t>Quel est le véritable prix à payer pour être un disciple de Jésus ? Cette étude sincère de 40 minutes examine les véritables exigences de la vie de disciple du Christ.</t>
+  </si>
+  <si>
+    <t>Êtes-vous à l'écoute de la voix de Jésus ? Cette étude de 40 minutes vous aide à reconnaître son appel et à y répondre.</t>
+  </si>
+  <si>
+    <t>Pourquoi Jésus est-il mort ? Que signifie la résurrection pour vous ? Cette étude de 40 minutes apporte des réponses claires qui changeront votre vie.</t>
+  </si>
+  <si>
+    <t>Jésus touchait les lépreux, les personnes brisées et les exclus. Cette réflexion de 40 minutes vous invite à faire l'expérience de son contact transformateur.</t>
+  </si>
+  <si>
+    <t>Que dit la Bible au sujet du paradis, de l'enfer et de la vie après la mort ? Cette étude de 40 minutes vous apporte des réponses claires et fondées sur la Bible.</t>
+  </si>
+  <si>
+    <t>La peur tient de nombreuses personnes sous son emprise. Découvrez ce que dit la Parole de Dieu et comment vous pouvez vous libérer de l'emprise de la peur.</t>
+  </si>
+  <si>
+    <t>À quoi ressemble une adoration authentique ? Cette étude de 40 minutes explore ce que signifie véritablement glorifier Dieu dans tous les domaines de la vie.</t>
+  </si>
+  <si>
+    <t>Le pardon peut briser l'emprise du passé. Cette étude de 40 minutes vous montre comment pardonner, à l'image de Dieu qui vous a pardonné.</t>
+  </si>
+  <si>
+    <t>Partez à la découverte du parcours d’Abraham, le père de la foi. Découvrez comment Dieu l’a appelé, l’a mis à l’épreuve et a tenu ses promesses. Une étude inspirante pour les enfants de 7 à 12 ans.</t>
+  </si>
+  <si>
+    <t>Plongez-vous dans Genèse 3 à 11 et découvrez les origines du péché, du déluge et des nations. Une étude découverte destinée aux enfants de 7 à 12 ans.</t>
+  </si>
+  <si>
+    <t>Jean 11-16 : Découvrez la puissance et l'amour incroyables de Jésus lorsqu'il ressuscite les morts, lave les pieds de ses disciples et leur promet le Saint-Esprit.</t>
+  </si>
+  <si>
+    <t>Jean 1–10 : Qui est Jésus ? Ce parcours de découverte destiné aux enfants de 7 à 12 ans met Jésus à l'honneur et laisse la Parole de Dieu parler d'elle-même.</t>
+  </si>
+  <si>
+    <t>Jean 17–21 : Suivre Jésus jusqu’à la croix, au tombeau vide et au-delà.
+Une étude biblique de découverte pour les enfants sur l’accomplissement du ministère de Jésus.</t>
+  </si>
+  <si>
+    <t>Genèse 1–2 : Explorez les merveilles de la création de Dieu avec cette étude biblique de découverte conçue pour les enfants de 7 à 12 ans.</t>
+  </si>
+  <si>
+    <t>Dieu est-il vraiment là ? Se soucie-t-il de vous ? Vous connaît-il ?
+Cette étude fondamentale aborde les questions les plus importantes de la vie.</t>
+  </si>
+  <si>
+    <t>Un parcours de 28 jours pour apprendre la méthode d’étude biblique inductive de Precept — Observez, Interprétez et Appliquez la Parole de Dieu par vous-même.</t>
+  </si>
+  <si>
+    <t>En 28 jours, apprenez à prier à travers la Parole de Dieu. Découvrez les principes de la prière tels qu’ils sont enseignés dans l’ensemble des Écritures.</t>
+  </si>
+  <si>
+    <t>Lorsque la vie soulève des questions difficiles, la Parole de Dieu apporte des réponses. Cette étude aborde certaines des questions les plus difficiles auxquelles les croyants sont confrontés.</t>
+  </si>
+  <si>
+    <t>Une étude approfondie des noms et du caractère de Dieu. Apprenez à Le connaître tel qu’Il est réellement, et non simplement tel que vous l’imaginez.</t>
+  </si>
+  <si>
+    <t>Étudiez les livres de Josué, des Juges et de Ruth et apprenez à choisir la victoire plutôt que la défaite dans votre marche quotidienne avec Dieu.</t>
+  </si>
+  <si>
+    <t>Une étude de Galates et d’Éphésiens. Découvrez la liberté que Christ a acquise pour vous et apprenez à vivre libres de l’esclavage du péché.</t>
+  </si>
+  <si>
+    <t>Une étude inductive de la Genèse, de l’Exode, du Lévitique, des Nombres et du Deutéronome. Découvrez les voies de Dieu et apprenez à y marcher.</t>
+  </si>
+  <si>
+    <t>Une étude inductive de l’Évangile selon Luc. Découvrez ce que signifie répondre à l’appel de Jésus à le suivre.</t>
+  </si>
+  <si>
+    <t>Hébreux : Qu’est-ce que la foi et comment vivre par la foi ? Étudiez la grande nuée de témoins et découvrez la supériorité de Christ.</t>
+  </si>
+  <si>
+    <t>Une étude « Saisir et Agir » (Seize and Apply) de l’épître aux Philippiens, avec environ 3 heures de travail personnel par semaine.</t>
+  </si>
+  <si>
+    <t>12;95 €</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="8" formatCode="#,##0.00\ &quot;€&quot;_);[Red]\(#,##0.00\ &quot;€&quot;\)"/>
+  </numFmts>
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -571,6 +423,20 @@
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -625,8 +491,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+  <cellXfs count="22">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -675,6 +541,21 @@
     <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="8" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="8" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -690,10 +571,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -894,20 +771,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G1000"/>
+  <dimension ref="A1:F1000"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.5" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="46" customWidth="1"/>
     <col min="3" max="3" width="28" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="10" customWidth="1"/>
-    <col min="6" max="6" width="55" customWidth="1"/>
-    <col min="7" max="7" width="15" customWidth="1"/>
-    <col min="8" max="26" width="8.6640625" customWidth="1"/>
+    <col min="5" max="5" width="55" customWidth="1"/>
+    <col min="6" max="6" width="15" customWidth="1"/>
+    <col min="7" max="25" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -926,897 +802,768 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="2" spans="1:6" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2"/>
       <c r="B2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>9</v>
+      <c r="D2" s="17">
+        <v>9.9499999999999993</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>60</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="5"/>
       <c r="B3" s="5" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>13</v>
+        <v>7</v>
+      </c>
+      <c r="D3" s="18">
+        <v>12.95</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="G3" s="7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>61</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2"/>
       <c r="B4" s="2" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>16</v>
+        <v>7</v>
+      </c>
+      <c r="D4" s="17">
+        <v>9.9499999999999993</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>62</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="5"/>
       <c r="B5" s="5" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>9</v>
+        <v>7</v>
+      </c>
+      <c r="D5" s="18">
+        <v>12.95</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>63</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
       <c r="B6" s="2" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>21</v>
+        <v>7</v>
+      </c>
+      <c r="D6" s="17">
+        <v>14.95</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>64</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="5"/>
       <c r="B7" s="5" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>16</v>
+        <v>7</v>
+      </c>
+      <c r="D7" s="18">
+        <v>12.95</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="G7" s="7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>65</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2"/>
       <c r="B8" s="2" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>26</v>
+        <v>7</v>
+      </c>
+      <c r="D8" s="17">
+        <v>12.95</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>66</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="5"/>
       <c r="B9" s="5" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>29</v>
+        <v>7</v>
+      </c>
+      <c r="D9" s="18">
+        <v>12.95</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>148</v>
-      </c>
-      <c r="G9" s="7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>67</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="2"/>
       <c r="B10" s="2" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>32</v>
+        <v>7</v>
+      </c>
+      <c r="D10" s="19" t="s">
+        <v>102</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="G10" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>68</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="5"/>
       <c r="B11" s="5" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>21</v>
+        <v>7</v>
+      </c>
+      <c r="D11" s="18">
+        <v>12.95</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="G11" s="7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>69</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="2"/>
       <c r="B12" s="2" t="s">
-        <v>36</v>
+        <v>18</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>21</v>
+        <v>7</v>
+      </c>
+      <c r="D12" s="17">
+        <v>12.95</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="G12" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>70</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="5"/>
       <c r="B13" s="5" t="s">
-        <v>38</v>
+        <v>19</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>39</v>
+        <v>7</v>
+      </c>
+      <c r="D13" s="18">
+        <v>9.9499999999999993</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="F13" s="5" t="s">
-        <v>152</v>
-      </c>
-      <c r="G13" s="7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>71</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="2"/>
       <c r="B14" s="2" t="s">
-        <v>41</v>
+        <v>21</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>39</v>
+        <v>22</v>
+      </c>
+      <c r="D14" s="17">
+        <v>6.95</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="G14" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>72</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="5"/>
       <c r="B15" s="5" t="s">
-        <v>44</v>
+        <v>23</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>39</v>
+        <v>22</v>
+      </c>
+      <c r="D15" s="18">
+        <v>6.95</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="F15" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="G15" s="7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>73</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="2"/>
       <c r="B16" s="2" t="s">
-        <v>47</v>
+        <v>24</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>39</v>
+        <v>22</v>
+      </c>
+      <c r="D16" s="17">
+        <v>6.95</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="G16" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>74</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="5"/>
       <c r="B17" s="5" t="s">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>39</v>
+        <v>22</v>
+      </c>
+      <c r="D17" s="18">
+        <v>6.95</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="F17" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="G17" s="7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>75</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="2"/>
       <c r="B18" s="2" t="s">
-        <v>53</v>
+        <v>26</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>39</v>
+        <v>22</v>
+      </c>
+      <c r="D18" s="17">
+        <v>6.95</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="G18" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>76</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="5"/>
       <c r="B19" s="5" t="s">
-        <v>56</v>
+        <v>27</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="D19" s="5" t="s">
-        <v>39</v>
+        <v>22</v>
+      </c>
+      <c r="D19" s="18">
+        <v>6.95</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="F19" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="G19" s="7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>77</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="2"/>
       <c r="B20" s="2" t="s">
-        <v>59</v>
+        <v>28</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>39</v>
+        <v>22</v>
+      </c>
+      <c r="D20" s="17">
+        <v>6.95</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="G20" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>78</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="5"/>
       <c r="B21" s="5" t="s">
-        <v>62</v>
+        <v>29</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="D21" s="5" t="s">
-        <v>39</v>
+        <v>22</v>
+      </c>
+      <c r="D21" s="18">
+        <v>6.95</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="F21" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="G21" s="7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>79</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="2"/>
       <c r="B22" s="2" t="s">
-        <v>65</v>
+        <v>30</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>39</v>
+        <v>22</v>
+      </c>
+      <c r="D22" s="17">
+        <v>6.95</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="G22" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>80</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="5"/>
       <c r="B23" s="5" t="s">
-        <v>68</v>
+        <v>31</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="D23" s="5" t="s">
-        <v>39</v>
+        <v>22</v>
+      </c>
+      <c r="D23" s="18">
+        <v>6.95</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="F23" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="G23" s="7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>81</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="2"/>
       <c r="B24" s="2" t="s">
-        <v>71</v>
+        <v>32</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>39</v>
+        <v>22</v>
+      </c>
+      <c r="D24" s="17">
+        <v>6.95</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="G24" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>82</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="5"/>
       <c r="B25" s="5" t="s">
-        <v>74</v>
+        <v>33</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="D25" s="5" t="s">
-        <v>39</v>
+        <v>22</v>
+      </c>
+      <c r="D25" s="18">
+        <v>6.95</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="F25" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="G25" s="7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>83</v>
+      </c>
+      <c r="F25" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="2"/>
       <c r="B26" s="2" t="s">
-        <v>77</v>
+        <v>34</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>39</v>
+        <v>22</v>
+      </c>
+      <c r="D26" s="17">
+        <v>6.95</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="G26" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>84</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="5"/>
       <c r="B27" s="5" t="s">
-        <v>80</v>
+        <v>35</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="D27" s="5" t="s">
-        <v>16</v>
+        <v>36</v>
+      </c>
+      <c r="D27" s="18">
+        <v>12.95</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="F27" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="G27" s="7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>85</v>
+      </c>
+      <c r="F27" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="2"/>
       <c r="B28" s="2" t="s">
-        <v>84</v>
+        <v>37</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>81</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>16</v>
+        <v>36</v>
+      </c>
+      <c r="D28" s="18">
+        <v>12.95</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="F28" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="G28" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F28" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="5"/>
       <c r="B29" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C29" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D29" s="18">
+        <v>12.95</v>
+      </c>
+      <c r="E29" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="C29" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="D29" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="E29" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="F29" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="G29" s="7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F29" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="2"/>
       <c r="B30" s="2" t="s">
-        <v>91</v>
+        <v>39</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>81</v>
-      </c>
-      <c r="D30" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D30" s="17">
+        <v>12.95</v>
+      </c>
+      <c r="E30" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="E30" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="F30" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="G30" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F30" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="5"/>
       <c r="B31" s="5" t="s">
-        <v>94</v>
+        <v>40</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="D31" s="5" t="s">
-        <v>88</v>
+        <v>36</v>
+      </c>
+      <c r="D31" s="18">
+        <v>12.95</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="F31" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="G31" s="7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>89</v>
+      </c>
+      <c r="F31" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="2"/>
       <c r="B32" s="2" t="s">
-        <v>97</v>
+        <v>41</v>
       </c>
       <c r="C32" s="11" t="s">
-        <v>81</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>16</v>
+        <v>36</v>
+      </c>
+      <c r="D32" s="18">
+        <v>12.95</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="F32" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="G32" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>90</v>
+      </c>
+      <c r="F32" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="5"/>
       <c r="B33" s="5" t="s">
-        <v>100</v>
+        <v>42</v>
       </c>
       <c r="C33" s="12" t="s">
-        <v>101</v>
-      </c>
-      <c r="D33" s="5" t="s">
-        <v>102</v>
+        <v>43</v>
+      </c>
+      <c r="D33" s="18">
+        <v>12.95</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="F33" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="G33" s="7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>91</v>
+      </c>
+      <c r="F33" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="2"/>
       <c r="B34" s="2" t="s">
-        <v>105</v>
+        <v>45</v>
       </c>
       <c r="C34" s="13" t="s">
-        <v>101</v>
-      </c>
-      <c r="D34" s="2" t="s">
-        <v>106</v>
+        <v>43</v>
+      </c>
+      <c r="D34" s="17">
+        <v>9.9499999999999993</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="F34" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="G34" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>92</v>
+      </c>
+      <c r="F34" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="5"/>
       <c r="B35" s="5" t="s">
-        <v>109</v>
+        <v>47</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>101</v>
-      </c>
-      <c r="D35" s="5" t="s">
-        <v>106</v>
+        <v>43</v>
+      </c>
+      <c r="D35" s="20" t="s">
+        <v>46</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="F35" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="G35" s="7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>93</v>
+      </c>
+      <c r="F35" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="2"/>
       <c r="B36" s="2" t="s">
-        <v>112</v>
+        <v>48</v>
       </c>
       <c r="C36" s="13" t="s">
-        <v>101</v>
-      </c>
-      <c r="D36" s="2" t="s">
-        <v>102</v>
+        <v>43</v>
+      </c>
+      <c r="D36" s="21" t="s">
+        <v>44</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="F36" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="G36" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>94</v>
+      </c>
+      <c r="F36" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="5"/>
       <c r="B37" s="5" t="s">
-        <v>115</v>
+        <v>49</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>101</v>
-      </c>
-      <c r="D37" s="5" t="s">
-        <v>116</v>
+        <v>43</v>
+      </c>
+      <c r="D37" s="18">
+        <v>12.95</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="F37" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="G37" s="7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>95</v>
+      </c>
+      <c r="F37" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="2"/>
       <c r="B38" s="2" t="s">
-        <v>119</v>
+        <v>50</v>
       </c>
       <c r="C38" s="14" t="s">
-        <v>120</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>39</v>
+        <v>51</v>
+      </c>
+      <c r="D38" s="17">
+        <v>9.9499999999999993</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="F38" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="G38" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>96</v>
+      </c>
+      <c r="F38" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="5"/>
       <c r="B39" s="5" t="s">
-        <v>123</v>
+        <v>52</v>
       </c>
       <c r="C39" s="15" t="s">
-        <v>120</v>
-      </c>
-      <c r="D39" s="5" t="s">
-        <v>39</v>
+        <v>51</v>
+      </c>
+      <c r="D39" s="18">
+        <v>9.9499999999999993</v>
       </c>
       <c r="E39" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="F39" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="G39" s="7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>97</v>
+      </c>
+      <c r="F39" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="2"/>
       <c r="B40" s="2" t="s">
-        <v>126</v>
+        <v>53</v>
       </c>
       <c r="C40" s="14" t="s">
-        <v>120</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>127</v>
+        <v>51</v>
+      </c>
+      <c r="D40" s="21" t="s">
+        <v>54</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="F40" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="G40" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>98</v>
+      </c>
+      <c r="F40" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="5"/>
       <c r="B41" s="5" t="s">
-        <v>130</v>
+        <v>55</v>
       </c>
       <c r="C41" s="15" t="s">
-        <v>120</v>
-      </c>
-      <c r="D41" s="5" t="s">
-        <v>39</v>
+        <v>51</v>
+      </c>
+      <c r="D41" s="20" t="s">
+        <v>20</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="F41" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="G41" s="7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>99</v>
+      </c>
+      <c r="F41" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="2"/>
       <c r="B42" s="2" t="s">
-        <v>133</v>
+        <v>56</v>
       </c>
       <c r="C42" s="14" t="s">
-        <v>120</v>
-      </c>
-      <c r="D42" s="2" t="s">
-        <v>39</v>
+        <v>51</v>
+      </c>
+      <c r="D42" s="21" t="s">
+        <v>20</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="F42" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="G42" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>100</v>
+      </c>
+      <c r="F42" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="5"/>
       <c r="B43" s="5" t="s">
-        <v>136</v>
+        <v>57</v>
       </c>
       <c r="C43" s="16" t="s">
-        <v>137</v>
-      </c>
-      <c r="D43" s="5" t="s">
-        <v>138</v>
+        <v>58</v>
+      </c>
+      <c r="D43" s="20" t="s">
+        <v>59</v>
       </c>
       <c r="E43" s="5" t="s">
-        <v>139</v>
-      </c>
-      <c r="F43" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="G43" s="7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="45" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="46" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="47" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="48" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+        <v>101</v>
+      </c>
+      <c r="F43" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="45" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="46" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="47" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="48" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="49" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="50" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="51" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -2771,50 +2518,56 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="G2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="G3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="G4" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="G5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="G6" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="G7" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="G8" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="G9" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="G10" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="G11" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="G12" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
-    <hyperlink ref="G13" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="G14" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="G15" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
-    <hyperlink ref="G16" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
-    <hyperlink ref="G17" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
-    <hyperlink ref="G18" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
-    <hyperlink ref="G19" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
-    <hyperlink ref="G20" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
-    <hyperlink ref="G21" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
-    <hyperlink ref="G22" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
-    <hyperlink ref="G23" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
-    <hyperlink ref="G24" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
-    <hyperlink ref="G25" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
-    <hyperlink ref="G26" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
-    <hyperlink ref="G27" r:id="rId26" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
-    <hyperlink ref="G28" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
-    <hyperlink ref="G29" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
-    <hyperlink ref="G30" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
-    <hyperlink ref="G31" r:id="rId30" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
-    <hyperlink ref="G32" r:id="rId31" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
-    <hyperlink ref="G33" r:id="rId32" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
-    <hyperlink ref="G34" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
-    <hyperlink ref="G35" r:id="rId34" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
-    <hyperlink ref="G36" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
-    <hyperlink ref="G37" r:id="rId36" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
-    <hyperlink ref="G38" r:id="rId37" xr:uid="{00000000-0004-0000-0000-000024000000}"/>
-    <hyperlink ref="G39" r:id="rId38" xr:uid="{00000000-0004-0000-0000-000025000000}"/>
-    <hyperlink ref="G40" r:id="rId39" xr:uid="{00000000-0004-0000-0000-000026000000}"/>
-    <hyperlink ref="G41" r:id="rId40" xr:uid="{00000000-0004-0000-0000-000027000000}"/>
-    <hyperlink ref="G42" r:id="rId41" xr:uid="{00000000-0004-0000-0000-000028000000}"/>
-    <hyperlink ref="G43" r:id="rId42" xr:uid="{00000000-0004-0000-0000-000029000000}"/>
+    <hyperlink ref="F2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="F3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="F4" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="F5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="F6" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="F7" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="F8" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="F9" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="F10" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="F11" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="F12" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="F13" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="F14" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="F15" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="F16" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="F17" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="F18" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="F19" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="F20" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="F21" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="F22" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="F23" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
+    <hyperlink ref="F24" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
+    <hyperlink ref="F25" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
+    <hyperlink ref="F26" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
+    <hyperlink ref="F27" r:id="rId26" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
+    <hyperlink ref="F28" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
+    <hyperlink ref="F29" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
+    <hyperlink ref="F30" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
+    <hyperlink ref="F31" r:id="rId30" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
+    <hyperlink ref="F32" r:id="rId31" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
+    <hyperlink ref="F33" r:id="rId32" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
+    <hyperlink ref="F34" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
+    <hyperlink ref="F35" r:id="rId34" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
+    <hyperlink ref="F36" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
+    <hyperlink ref="F37" r:id="rId36" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
+    <hyperlink ref="F38" r:id="rId37" xr:uid="{00000000-0004-0000-0000-000024000000}"/>
+    <hyperlink ref="F39" r:id="rId38" xr:uid="{00000000-0004-0000-0000-000025000000}"/>
+    <hyperlink ref="F40" r:id="rId39" xr:uid="{00000000-0004-0000-0000-000026000000}"/>
+    <hyperlink ref="F41" r:id="rId40" xr:uid="{00000000-0004-0000-0000-000027000000}"/>
+    <hyperlink ref="F42" r:id="rId41" xr:uid="{00000000-0004-0000-0000-000028000000}"/>
+    <hyperlink ref="F43" r:id="rId42" xr:uid="{00000000-0004-0000-0000-000029000000}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{80c03608-5f64-40bb-9c70-9394abe6011c}" enabled="0" method="" siteId="{80c03608-5f64-40bb-9c70-9394abe6011c}" removed="1"/>
+</clbl:labelList>
 </file>
</xml_diff>